<commit_message>
minor work, updates to shopping list
</commit_message>
<xml_diff>
--- a/shopping/24AUGUST_A.xlsx
+++ b/shopping/24AUGUST_A.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\asiadel\Documents\FIRO\firo_electronics\shopping\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FBFE05B-6C60-453D-8C43-D7D71B556FFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EFBBE17-6E84-4C55-8022-891E88A9E6D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="181">
   <si>
     <t>Name</t>
   </si>
@@ -84,9 +84,6 @@
   </si>
   <si>
     <t>https://de.farnell.com/en-DE/diodes-inc/2n7002k-7/mosfet-n-ch-60v-0-3a-sot-23/dp/1713825</t>
-  </si>
-  <si>
-    <t>https://de.farnell.com/en-DE/vishay/vj0805y104kxamt/cap-0-1-f-50v-10-x7r-0805/dp/2896746</t>
   </si>
   <si>
     <t>MURATA GRT21BR71H474KE01L</t>
@@ -134,9 +131,6 @@
   </si>
   <si>
     <t>MLCC, 0.33 µF, 50 V, 0805, ± 10%, X7R</t>
-  </si>
-  <si>
-    <t>https://de.farnell.com/en-DE/vishay/vj0805a102gxxpw1bc/cap-1000pf-25v-2-c0g-np0-0805/dp/2896470</t>
   </si>
   <si>
     <t>WALSIN WF12P1201FTL</t>
@@ -614,6 +608,9 @@
   </si>
   <si>
     <t>https://de.farnell.com/en-DE/vishay/sidr392dp-t1-ge3/mosfet-n-ch-30v-100a-150deg-c/dp/2932895</t>
+  </si>
+  <si>
+    <t>https://de.farnell.com/en-DE/yageo/cs0805kkx7r0bb104/cap-0-1uf-100v-mlcc-0805/dp/3369404</t>
   </si>
 </sst>
 </file>
@@ -1091,10 +1088,10 @@
       </c>
       <c r="G1" s="1"/>
       <c r="H1" s="1" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="J1" s="1"/>
     </row>
@@ -1134,13 +1131,13 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="C3" s="12" t="s">
         <v>84</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="C3" s="12" t="s">
-        <v>86</v>
       </c>
       <c r="D3" s="10">
         <v>0.41799999999999998</v>
@@ -1202,13 +1199,13 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="C5" s="12" t="s">
         <v>81</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="C5" s="12" t="s">
-        <v>83</v>
       </c>
       <c r="D5" s="10">
         <v>1.1299999999999999</v>
@@ -1236,13 +1233,13 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="C6" s="12" t="s">
         <v>99</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="C6" s="12" t="s">
-        <v>101</v>
       </c>
       <c r="D6" s="10">
         <v>9.34</v>
@@ -1270,13 +1267,13 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="C7" s="15" t="s">
         <v>93</v>
-      </c>
-      <c r="B7" s="14" t="s">
-        <v>94</v>
-      </c>
-      <c r="C7" s="15" t="s">
-        <v>95</v>
       </c>
       <c r="D7" s="16">
         <v>0.68899999999999995</v>
@@ -1304,13 +1301,13 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="C8" s="15" t="s">
         <v>90</v>
-      </c>
-      <c r="B8" s="14" t="s">
-        <v>91</v>
-      </c>
-      <c r="C8" s="15" t="s">
-        <v>92</v>
       </c>
       <c r="D8" s="16">
         <v>0.27500000000000002</v>
@@ -1338,13 +1335,13 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="C9" s="15" t="s">
         <v>96</v>
-      </c>
-      <c r="B9" s="14" t="s">
-        <v>97</v>
-      </c>
-      <c r="C9" s="15" t="s">
-        <v>98</v>
       </c>
       <c r="D9" s="16">
         <v>0.75</v>
@@ -1372,13 +1369,13 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="C10" s="15" t="s">
         <v>87</v>
-      </c>
-      <c r="B10" s="14" t="s">
-        <v>88</v>
-      </c>
-      <c r="C10" s="15" t="s">
-        <v>89</v>
       </c>
       <c r="D10" s="16">
         <v>0.35299999999999998</v>
@@ -1440,13 +1437,13 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="B12" s="14" t="s">
+        <v>178</v>
+      </c>
+      <c r="C12" s="35" t="s">
         <v>179</v>
-      </c>
-      <c r="B12" s="14" t="s">
-        <v>180</v>
-      </c>
-      <c r="C12" s="35" t="s">
-        <v>181</v>
       </c>
       <c r="D12" s="16">
         <v>1.46</v>
@@ -1474,13 +1471,13 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="C13" s="6" t="s">
         <v>25</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>26</v>
       </c>
       <c r="D13" s="4">
         <v>0.121</v>
@@ -1499,7 +1496,7 @@
         <v>10</v>
       </c>
       <c r="I13" s="3">
-        <f>D13*H13</f>
+        <f t="shared" ref="I13:I22" si="4">D13*H13</f>
         <v>1.21</v>
       </c>
       <c r="J13" s="3" t="s">
@@ -1508,13 +1505,13 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D14" s="4">
         <v>9.7000000000000003E-2</v>
@@ -1533,7 +1530,7 @@
         <v>10</v>
       </c>
       <c r="I14" s="3">
-        <f>D14*H14</f>
+        <f t="shared" si="4"/>
         <v>0.97</v>
       </c>
       <c r="J14" s="3" t="s">
@@ -1542,13 +1539,13 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D15" s="4">
         <v>0.115</v>
@@ -1567,7 +1564,7 @@
         <v>10</v>
       </c>
       <c r="I15" s="3">
-        <f>D15*H15</f>
+        <f t="shared" si="4"/>
         <v>1.1500000000000001</v>
       </c>
       <c r="J15" s="3" t="s">
@@ -1576,13 +1573,13 @@
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="C16" s="6" t="s">
         <v>105</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>107</v>
       </c>
       <c r="D16" s="3">
         <v>4.8000000000000001E-2</v>
@@ -1601,7 +1598,7 @@
         <v>10</v>
       </c>
       <c r="I16" s="3">
-        <f>D16*H16</f>
+        <f t="shared" si="4"/>
         <v>0.48</v>
       </c>
       <c r="J16" s="3" t="s">
@@ -1610,23 +1607,23 @@
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>16</v>
+        <v>180</v>
       </c>
       <c r="D17" s="4">
-        <v>0.17499999999999999</v>
+        <v>0.108</v>
       </c>
       <c r="E17" s="3">
         <v>2</v>
       </c>
       <c r="F17" s="5">
         <f t="shared" si="3"/>
-        <v>0.35</v>
+        <v>0.216</v>
       </c>
       <c r="G17" s="3" t="s">
         <v>9</v>
@@ -1635,8 +1632,8 @@
         <v>5</v>
       </c>
       <c r="I17" s="3">
-        <f>D17*H17</f>
-        <v>0.875</v>
+        <f t="shared" si="4"/>
+        <v>0.54</v>
       </c>
       <c r="J17" s="3" t="s">
         <v>9</v>
@@ -1644,23 +1641,23 @@
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B18" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B18" s="3" t="s">
-        <v>28</v>
-      </c>
       <c r="C18" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D18" s="4">
-        <v>0.121</v>
+        <v>0.13500000000000001</v>
       </c>
       <c r="E18" s="3">
         <v>1</v>
       </c>
       <c r="F18" s="5">
         <f t="shared" si="3"/>
-        <v>0.121</v>
+        <v>0.13500000000000001</v>
       </c>
       <c r="G18" s="3" t="s">
         <v>9</v>
@@ -1669,8 +1666,8 @@
         <v>10</v>
       </c>
       <c r="I18" s="3">
-        <f>D18*H18</f>
-        <v>1.21</v>
+        <f t="shared" si="4"/>
+        <v>1.35</v>
       </c>
       <c r="J18" s="3" t="s">
         <v>9</v>
@@ -1678,13 +1675,13 @@
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="C19" s="6" t="s">
         <v>18</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>19</v>
       </c>
       <c r="D19" s="4">
         <v>0.13100000000000001</v>
@@ -1703,7 +1700,7 @@
         <v>5</v>
       </c>
       <c r="I19" s="3">
-        <f>D19*H19</f>
+        <f t="shared" si="4"/>
         <v>0.65500000000000003</v>
       </c>
       <c r="J19" s="3" t="s">
@@ -1712,13 +1709,13 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="C20" s="6" t="s">
         <v>108</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>110</v>
       </c>
       <c r="D20" s="4">
         <v>0.126</v>
@@ -1737,7 +1734,7 @@
         <v>5</v>
       </c>
       <c r="I20" s="3">
-        <f>D20*H20</f>
+        <f t="shared" si="4"/>
         <v>0.63</v>
       </c>
       <c r="J20" s="3" t="s">
@@ -1746,13 +1743,13 @@
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="C21" s="6" t="s">
         <v>102</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>104</v>
       </c>
       <c r="D21" s="4">
         <v>0.159</v>
@@ -1771,7 +1768,7 @@
         <v>10</v>
       </c>
       <c r="I21" s="3">
-        <f>D21*H21</f>
+        <f t="shared" si="4"/>
         <v>1.59</v>
       </c>
       <c r="J21" s="3" t="s">
@@ -1780,13 +1777,13 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="C22" s="6" t="s">
         <v>111</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="C22" s="6" t="s">
-        <v>113</v>
       </c>
       <c r="D22" s="4">
         <v>8.2000000000000003E-2</v>
@@ -1805,7 +1802,7 @@
         <v>5</v>
       </c>
       <c r="I22" s="3">
-        <f>D22*H22</f>
+        <f t="shared" si="4"/>
         <v>0.41000000000000003</v>
       </c>
       <c r="J22" s="3" t="s">
@@ -1814,13 +1811,13 @@
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D23" s="4">
         <v>4.0999999999999996</v>
@@ -1839,7 +1836,7 @@
         <v>1</v>
       </c>
       <c r="I23" s="3">
-        <f t="shared" ref="I23" si="4">D23*H23</f>
+        <f t="shared" ref="I23" si="5">D23*H23</f>
         <v>4.0999999999999996</v>
       </c>
       <c r="J23" s="3" t="s">
@@ -1848,13 +1845,13 @@
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B24" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B24" s="3" t="s">
-        <v>21</v>
-      </c>
       <c r="C24" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D24" s="4">
         <v>0.48199999999999998</v>
@@ -1873,7 +1870,7 @@
         <v>5</v>
       </c>
       <c r="I24" s="3">
-        <f>D24*H24</f>
+        <f t="shared" ref="I24:I42" si="6">D24*H24</f>
         <v>2.41</v>
       </c>
       <c r="J24" s="3" t="s">
@@ -1882,13 +1879,13 @@
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D25" s="4">
         <v>0.90600000000000003</v>
@@ -1907,7 +1904,7 @@
         <v>1</v>
       </c>
       <c r="I25" s="3">
-        <f>D25*H25</f>
+        <f t="shared" si="6"/>
         <v>0.90600000000000003</v>
       </c>
       <c r="J25" s="3" t="s">
@@ -1916,13 +1913,13 @@
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C26" s="6" t="s">
         <v>129</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="C26" s="6" t="s">
-        <v>131</v>
       </c>
       <c r="D26" s="4">
         <v>2.7E-2</v>
@@ -1941,7 +1938,7 @@
         <v>10</v>
       </c>
       <c r="I26" s="3">
-        <f>D26*H26</f>
+        <f t="shared" si="6"/>
         <v>0.27</v>
       </c>
       <c r="J26" s="3" t="s">
@@ -1950,13 +1947,13 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C27" s="6" t="s">
         <v>120</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="C27" s="6" t="s">
-        <v>122</v>
       </c>
       <c r="D27" s="4">
         <v>2.5000000000000001E-2</v>
@@ -1975,7 +1972,7 @@
         <v>10</v>
       </c>
       <c r="I27" s="3">
-        <f>D27*H27</f>
+        <f t="shared" si="6"/>
         <v>0.25</v>
       </c>
       <c r="J27" s="3" t="s">
@@ -1984,13 +1981,13 @@
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C28" s="6" t="s">
         <v>33</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="C28" s="6" t="s">
-        <v>35</v>
       </c>
       <c r="D28" s="4">
         <v>7.0000000000000007E-2</v>
@@ -2009,7 +2006,7 @@
         <v>10</v>
       </c>
       <c r="I28" s="3">
-        <f>D28*H28</f>
+        <f t="shared" si="6"/>
         <v>0.70000000000000007</v>
       </c>
       <c r="J28" s="3" t="s">
@@ -2018,13 +2015,13 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C29" s="6" t="s">
         <v>117</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="C29" s="6" t="s">
-        <v>119</v>
       </c>
       <c r="D29" s="4">
         <v>8.8999999999999996E-2</v>
@@ -2043,7 +2040,7 @@
         <v>10</v>
       </c>
       <c r="I29" s="3">
-        <f>D29*H29</f>
+        <f t="shared" si="6"/>
         <v>0.8899999999999999</v>
       </c>
       <c r="J29" s="3" t="s">
@@ -2052,13 +2049,13 @@
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C30" s="6" t="s">
         <v>30</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="C30" s="6" t="s">
-        <v>32</v>
       </c>
       <c r="D30" s="4">
         <v>0.13500000000000001</v>
@@ -2077,7 +2074,7 @@
         <v>10</v>
       </c>
       <c r="I30" s="3">
-        <f>D30*H30</f>
+        <f t="shared" si="6"/>
         <v>1.35</v>
       </c>
       <c r="J30" s="3" t="s">
@@ -2086,13 +2083,13 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C31" s="6" t="s">
         <v>54</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C31" s="6" t="s">
-        <v>56</v>
       </c>
       <c r="D31" s="4">
         <v>1.9E-2</v>
@@ -2111,7 +2108,7 @@
         <v>10</v>
       </c>
       <c r="I31" s="3">
-        <f>D31*H31</f>
+        <f t="shared" si="6"/>
         <v>0.19</v>
       </c>
       <c r="J31" s="3" t="s">
@@ -2120,13 +2117,13 @@
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C32" s="6" t="s">
         <v>51</v>
-      </c>
-      <c r="B32" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="C32" s="6" t="s">
-        <v>53</v>
       </c>
       <c r="D32" s="4">
         <v>4.7E-2</v>
@@ -2145,7 +2142,7 @@
         <v>10</v>
       </c>
       <c r="I32" s="3">
-        <f>D32*H32</f>
+        <f t="shared" si="6"/>
         <v>0.47</v>
       </c>
       <c r="J32" s="3" t="s">
@@ -2154,13 +2151,13 @@
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="D33" s="4">
         <v>2.8000000000000001E-2</v>
@@ -2179,7 +2176,7 @@
         <v>10</v>
       </c>
       <c r="I33" s="3">
-        <f>D33*H33</f>
+        <f t="shared" si="6"/>
         <v>0.28000000000000003</v>
       </c>
       <c r="J33" s="3" t="s">
@@ -2188,13 +2185,13 @@
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C34" s="6" t="s">
         <v>57</v>
-      </c>
-      <c r="B34" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="C34" s="6" t="s">
-        <v>59</v>
       </c>
       <c r="D34" s="4">
         <v>0.1</v>
@@ -2213,7 +2210,7 @@
         <v>10</v>
       </c>
       <c r="I34" s="3">
-        <f>D34*H34</f>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="J34" s="3" t="s">
@@ -2222,13 +2219,13 @@
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C35" s="6" t="s">
         <v>126</v>
-      </c>
-      <c r="B35" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="C35" s="6" t="s">
-        <v>128</v>
       </c>
       <c r="D35" s="4">
         <v>5.0999999999999997E-2</v>
@@ -2247,7 +2244,7 @@
         <v>10</v>
       </c>
       <c r="I35" s="3">
-        <f>D35*H35</f>
+        <f t="shared" si="6"/>
         <v>0.51</v>
       </c>
       <c r="J35" s="3" t="s">
@@ -2256,13 +2253,13 @@
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="C36" s="6" t="s">
         <v>123</v>
-      </c>
-      <c r="B36" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="C36" s="6" t="s">
-        <v>125</v>
       </c>
       <c r="D36" s="4">
         <v>4.5999999999999999E-2</v>
@@ -2281,7 +2278,7 @@
         <v>10</v>
       </c>
       <c r="I36" s="3">
-        <f>D36*H36</f>
+        <f t="shared" si="6"/>
         <v>0.45999999999999996</v>
       </c>
       <c r="J36" s="3" t="s">
@@ -2290,13 +2287,13 @@
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C37" s="6" t="s">
         <v>39</v>
-      </c>
-      <c r="B37" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C37" s="6" t="s">
-        <v>41</v>
       </c>
       <c r="D37" s="4">
         <v>8.8999999999999996E-2</v>
@@ -2315,7 +2312,7 @@
         <v>10</v>
       </c>
       <c r="I37" s="3">
-        <f>D37*H37</f>
+        <f t="shared" si="6"/>
         <v>0.8899999999999999</v>
       </c>
       <c r="J37" s="3" t="s">
@@ -2324,13 +2321,13 @@
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="C38" s="6" t="s">
         <v>114</v>
-      </c>
-      <c r="B38" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="C38" s="6" t="s">
-        <v>116</v>
       </c>
       <c r="D38" s="4">
         <v>2.9000000000000001E-2</v>
@@ -2349,7 +2346,7 @@
         <v>10</v>
       </c>
       <c r="I38" s="3">
-        <f>D38*H38</f>
+        <f t="shared" si="6"/>
         <v>0.29000000000000004</v>
       </c>
       <c r="J38" s="3" t="s">
@@ -2358,13 +2355,13 @@
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C39" s="6" t="s">
         <v>42</v>
-      </c>
-      <c r="B39" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="C39" s="6" t="s">
-        <v>44</v>
       </c>
       <c r="D39" s="4">
         <v>2.7E-2</v>
@@ -2383,7 +2380,7 @@
         <v>10</v>
       </c>
       <c r="I39" s="3">
-        <f>D39*H39</f>
+        <f t="shared" si="6"/>
         <v>0.27</v>
       </c>
       <c r="J39" s="3" t="s">
@@ -2392,13 +2389,13 @@
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C40" s="6" t="s">
         <v>36</v>
-      </c>
-      <c r="B40" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C40" s="6" t="s">
-        <v>38</v>
       </c>
       <c r="D40" s="4">
         <v>6.2E-2</v>
@@ -2417,7 +2414,7 @@
         <v>10</v>
       </c>
       <c r="I40" s="3">
-        <f>D40*H40</f>
+        <f t="shared" si="6"/>
         <v>0.62</v>
       </c>
       <c r="J40" s="3" t="s">
@@ -2426,13 +2423,13 @@
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C41" s="6" t="s">
         <v>48</v>
-      </c>
-      <c r="B41" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="C41" s="6" t="s">
-        <v>50</v>
       </c>
       <c r="D41" s="4">
         <v>1.9E-2</v>
@@ -2451,7 +2448,7 @@
         <v>10</v>
       </c>
       <c r="I41" s="3">
-        <f>D41*H41</f>
+        <f t="shared" si="6"/>
         <v>0.19</v>
       </c>
       <c r="J41" s="3" t="s">
@@ -2460,13 +2457,13 @@
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C42" s="6" t="s">
         <v>45</v>
-      </c>
-      <c r="B42" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C42" s="6" t="s">
-        <v>47</v>
       </c>
       <c r="D42" s="4">
         <v>2.7E-2</v>
@@ -2485,7 +2482,7 @@
         <v>10</v>
       </c>
       <c r="I42" s="3">
-        <f>D42*H42</f>
+        <f t="shared" si="6"/>
         <v>0.27</v>
       </c>
       <c r="J42" s="3" t="s">
@@ -2494,13 +2491,13 @@
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A43" s="18" t="s">
+        <v>144</v>
+      </c>
+      <c r="B43" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="C43" s="20" t="s">
         <v>146</v>
-      </c>
-      <c r="B43" s="19" t="s">
-        <v>147</v>
-      </c>
-      <c r="C43" s="20" t="s">
-        <v>148</v>
       </c>
       <c r="D43" s="21">
         <v>0.52600000000000002</v>
@@ -2519,7 +2516,7 @@
         <v>10</v>
       </c>
       <c r="I43" s="19">
-        <f t="shared" ref="I43:I58" si="5">D43*H43</f>
+        <f t="shared" ref="I43:I58" si="7">D43*H43</f>
         <v>5.26</v>
       </c>
       <c r="J43" s="19" t="s">
@@ -2528,13 +2525,13 @@
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A44" s="18" t="s">
+        <v>147</v>
+      </c>
+      <c r="B44" s="19" t="s">
+        <v>148</v>
+      </c>
+      <c r="C44" s="20" t="s">
         <v>149</v>
-      </c>
-      <c r="B44" s="19" t="s">
-        <v>150</v>
-      </c>
-      <c r="C44" s="20" t="s">
-        <v>151</v>
       </c>
       <c r="D44" s="21">
         <v>0.78800000000000003</v>
@@ -2553,7 +2550,7 @@
         <v>2</v>
       </c>
       <c r="I44" s="19">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1.5760000000000001</v>
       </c>
       <c r="J44" s="19" t="s">
@@ -2562,13 +2559,13 @@
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A45" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="B45" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="C45" s="20" t="s">
         <v>60</v>
-      </c>
-      <c r="B45" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="C45" s="20" t="s">
-        <v>62</v>
       </c>
       <c r="D45" s="21">
         <v>0.85</v>
@@ -2587,7 +2584,7 @@
         <v>1</v>
       </c>
       <c r="I45" s="19">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0.85</v>
       </c>
       <c r="J45" s="19" t="s">
@@ -2596,13 +2593,13 @@
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A46" s="18" t="s">
+        <v>150</v>
+      </c>
+      <c r="B46" s="19" t="s">
+        <v>151</v>
+      </c>
+      <c r="C46" s="20" t="s">
         <v>152</v>
-      </c>
-      <c r="B46" s="19" t="s">
-        <v>153</v>
-      </c>
-      <c r="C46" s="20" t="s">
-        <v>154</v>
       </c>
       <c r="D46" s="21">
         <v>0.495</v>
@@ -2621,7 +2618,7 @@
         <v>1</v>
       </c>
       <c r="I46" s="19">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0.495</v>
       </c>
       <c r="J46" s="19" t="s">
@@ -2630,13 +2627,13 @@
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A47" s="18" t="s">
+        <v>153</v>
+      </c>
+      <c r="B47" s="19" t="s">
+        <v>154</v>
+      </c>
+      <c r="C47" s="20" t="s">
         <v>155</v>
-      </c>
-      <c r="B47" s="19" t="s">
-        <v>156</v>
-      </c>
-      <c r="C47" s="20" t="s">
-        <v>157</v>
       </c>
       <c r="D47" s="21">
         <v>0.59799999999999998</v>
@@ -2655,7 +2652,7 @@
         <v>1</v>
       </c>
       <c r="I47" s="19">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0.59799999999999998</v>
       </c>
       <c r="J47" s="19" t="s">
@@ -2664,13 +2661,13 @@
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A48" s="18" t="s">
+        <v>156</v>
+      </c>
+      <c r="B48" s="19" t="s">
+        <v>157</v>
+      </c>
+      <c r="C48" s="20" t="s">
         <v>158</v>
-      </c>
-      <c r="B48" s="19" t="s">
-        <v>159</v>
-      </c>
-      <c r="C48" s="20" t="s">
-        <v>160</v>
       </c>
       <c r="D48" s="21">
         <v>0.56799999999999995</v>
@@ -2689,7 +2686,7 @@
         <v>1</v>
       </c>
       <c r="I48" s="19">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0.56799999999999995</v>
       </c>
       <c r="J48" s="19" t="s">
@@ -2698,13 +2695,13 @@
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A49" s="18" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B49" s="19" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C49" s="20" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D49" s="21">
         <v>3.22</v>
@@ -2723,7 +2720,7 @@
         <v>2</v>
       </c>
       <c r="I49" s="19">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>6.44</v>
       </c>
       <c r="J49" s="19" t="s">
@@ -2732,13 +2729,13 @@
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A50" s="18" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B50" s="19" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C50" s="20" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="D50" s="21">
         <v>4.1399999999999997</v>
@@ -2757,7 +2754,7 @@
         <v>1</v>
       </c>
       <c r="I50" s="19">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>4.1399999999999997</v>
       </c>
       <c r="J50" s="19" t="s">
@@ -2766,13 +2763,13 @@
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A51" s="18" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B51" s="19" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C51" s="20" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="D51" s="21">
         <v>4.99</v>
@@ -2791,7 +2788,7 @@
         <v>3</v>
       </c>
       <c r="I51" s="19">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>14.97</v>
       </c>
       <c r="J51" s="19" t="s">
@@ -2800,13 +2797,13 @@
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A52" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="B52" s="19" t="s">
+        <v>62</v>
+      </c>
+      <c r="C52" s="20" t="s">
         <v>63</v>
-      </c>
-      <c r="B52" s="19" t="s">
-        <v>64</v>
-      </c>
-      <c r="C52" s="20" t="s">
-        <v>65</v>
       </c>
       <c r="D52" s="21">
         <v>0.95</v>
@@ -2833,13 +2830,13 @@
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A53" s="23" t="s">
+        <v>64</v>
+      </c>
+      <c r="B53" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="C53" s="25" t="s">
         <v>66</v>
-      </c>
-      <c r="B53" s="24" t="s">
-        <v>67</v>
-      </c>
-      <c r="C53" s="25" t="s">
-        <v>68</v>
       </c>
       <c r="D53" s="26">
         <v>0.16800000000000001</v>
@@ -2858,7 +2855,7 @@
         <v>5</v>
       </c>
       <c r="I53" s="24">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0.84000000000000008</v>
       </c>
       <c r="J53" s="24" t="s">
@@ -2867,13 +2864,13 @@
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A54" s="23" t="s">
+        <v>67</v>
+      </c>
+      <c r="B54" s="24" t="s">
+        <v>68</v>
+      </c>
+      <c r="C54" s="25" t="s">
         <v>69</v>
-      </c>
-      <c r="B54" s="24" t="s">
-        <v>70</v>
-      </c>
-      <c r="C54" s="25" t="s">
-        <v>71</v>
       </c>
       <c r="D54" s="26">
         <v>0.125</v>
@@ -2892,7 +2889,7 @@
         <v>6</v>
       </c>
       <c r="I54" s="24">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0.75</v>
       </c>
       <c r="J54" s="24" t="s">
@@ -2901,13 +2898,13 @@
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A55" s="28" t="s">
+        <v>70</v>
+      </c>
+      <c r="B55" s="29" t="s">
+        <v>71</v>
+      </c>
+      <c r="C55" s="30" t="s">
         <v>72</v>
-      </c>
-      <c r="B55" s="29" t="s">
-        <v>73</v>
-      </c>
-      <c r="C55" s="30" t="s">
-        <v>74</v>
       </c>
       <c r="D55" s="31">
         <v>0.82799999999999996</v>
@@ -2926,7 +2923,7 @@
         <v>2</v>
       </c>
       <c r="I55" s="29">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1.6559999999999999</v>
       </c>
       <c r="J55" s="29" t="s">
@@ -2935,13 +2932,13 @@
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A56" s="28" t="s">
+        <v>165</v>
+      </c>
+      <c r="B56" s="29" t="s">
+        <v>166</v>
+      </c>
+      <c r="C56" s="30" t="s">
         <v>167</v>
-      </c>
-      <c r="B56" s="29" t="s">
-        <v>168</v>
-      </c>
-      <c r="C56" s="30" t="s">
-        <v>169</v>
       </c>
       <c r="D56" s="31">
         <v>0.33400000000000002</v>
@@ -2960,7 +2957,7 @@
         <v>10</v>
       </c>
       <c r="I56" s="29">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>3.3400000000000003</v>
       </c>
       <c r="J56" s="29" t="s">
@@ -2969,13 +2966,13 @@
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A57" s="28" t="s">
+        <v>73</v>
+      </c>
+      <c r="B57" s="29" t="s">
+        <v>74</v>
+      </c>
+      <c r="C57" s="30" t="s">
         <v>75</v>
-      </c>
-      <c r="B57" s="29" t="s">
-        <v>76</v>
-      </c>
-      <c r="C57" s="30" t="s">
-        <v>77</v>
       </c>
       <c r="D57" s="31">
         <v>1.29</v>
@@ -2994,7 +2991,7 @@
         <v>1</v>
       </c>
       <c r="I57" s="29">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1.29</v>
       </c>
       <c r="J57" s="29" t="s">
@@ -3003,13 +3000,13 @@
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A58" s="28" t="s">
+        <v>76</v>
+      </c>
+      <c r="B58" s="29" t="s">
+        <v>77</v>
+      </c>
+      <c r="C58" s="30" t="s">
         <v>78</v>
-      </c>
-      <c r="B58" s="29" t="s">
-        <v>79</v>
-      </c>
-      <c r="C58" s="30" t="s">
-        <v>80</v>
       </c>
       <c r="D58" s="31">
         <v>0.36699999999999999</v>
@@ -3028,7 +3025,7 @@
         <v>1</v>
       </c>
       <c r="I58" s="29">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>0.36699999999999999</v>
       </c>
       <c r="J58" s="29" t="s">
@@ -3037,21 +3034,21 @@
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.35">
       <c r="E59" s="33" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F59" s="34">
         <f>SUM(F2:F58)</f>
-        <v>71.614000000000033</v>
+        <v>71.494000000000028</v>
       </c>
       <c r="G59" s="33" t="s">
         <v>9</v>
       </c>
       <c r="H59" s="33" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="I59" s="33">
         <f>SUM(I2:I58)</f>
-        <v>100.16900000000003</v>
+        <v>99.974000000000032</v>
       </c>
       <c r="J59" s="33" t="s">
         <v>9</v>
@@ -3083,30 +3080,28 @@
     <hyperlink ref="C42" r:id="rId22" xr:uid="{C7DE7188-4BD3-4132-BC36-097E1D03FD84}"/>
     <hyperlink ref="C41" r:id="rId23" xr:uid="{1949DB4B-E2C3-436B-9AE3-791997D69328}"/>
     <hyperlink ref="C31" r:id="rId24" xr:uid="{6CC8A787-209A-453C-AB0C-010F171ACDA7}"/>
-    <hyperlink ref="C18" r:id="rId25" display="https://de.farnell.com/en-DE/vishay/vj0805a102gxxpw1bc/cap-1000pf-25v-2-c0g-np0-0805/dp/2896469" xr:uid="{90B9806A-71AA-46B3-A840-C35BEE7D553B}"/>
-    <hyperlink ref="C17" r:id="rId26" xr:uid="{82FE9AB9-F5F5-44C2-9F1F-B4FAF305AF7E}"/>
-    <hyperlink ref="C43" r:id="rId27" xr:uid="{3682C2B1-4476-4430-8109-2353A524C137}"/>
-    <hyperlink ref="C52" r:id="rId28" xr:uid="{4E741034-1394-42D0-8739-142B2406FCB0}"/>
-    <hyperlink ref="C45" r:id="rId29" xr:uid="{B384043F-23E3-43F1-862B-A7356F8867EC}"/>
-    <hyperlink ref="C53" r:id="rId30" xr:uid="{6E3DD45A-D91A-4A36-BF25-EEBD7F10DAE9}"/>
-    <hyperlink ref="C54" r:id="rId31" xr:uid="{6453CA4A-2AC9-4105-BF0F-FBCA99EEB8D1}"/>
-    <hyperlink ref="C55" r:id="rId32" xr:uid="{AA389CBE-2BA8-4629-8201-C6131E27DFBE}"/>
-    <hyperlink ref="C57" r:id="rId33" xr:uid="{6F0FC5B8-F6F6-4C15-BB76-EAAC8F1ACA1A}"/>
-    <hyperlink ref="C58" r:id="rId34" xr:uid="{567094FA-4502-4190-8663-26683FDE48C7}"/>
-    <hyperlink ref="C14" r:id="rId35" xr:uid="{A74EF970-0D7C-46E9-AC9F-E64E0416DCED}"/>
-    <hyperlink ref="C15" r:id="rId36" xr:uid="{4119277E-53BD-480A-AAD0-5BF01C147C02}"/>
-    <hyperlink ref="C16" r:id="rId37" xr:uid="{F67B1A2A-4358-43B4-86C7-5A00503AFF4C}"/>
-    <hyperlink ref="C21" r:id="rId38" xr:uid="{D337D021-F911-411B-BC13-9CBEF73345EF}"/>
-    <hyperlink ref="C25" r:id="rId39" xr:uid="{740D5D52-5E21-47B4-AE24-5AD4FADFC13D}"/>
-    <hyperlink ref="C26" r:id="rId40" xr:uid="{1E8B1C6A-A129-4E2E-9CF9-FFC3608F8F60}"/>
-    <hyperlink ref="C27" r:id="rId41" xr:uid="{F9D674A4-D18C-4CA7-BDBD-994C52816696}"/>
-    <hyperlink ref="C30" r:id="rId42" xr:uid="{C0358119-16A3-40A0-ACE5-D9B3CA1113E8}"/>
-    <hyperlink ref="C33" r:id="rId43" xr:uid="{17934D35-BFF5-473B-9CF6-081553A57DB8}"/>
-    <hyperlink ref="C34" r:id="rId44" xr:uid="{C23108EC-6E51-4B52-BFBF-0ECFFE00B2CC}"/>
-    <hyperlink ref="C35" r:id="rId45" xr:uid="{58BEF89A-A2C4-4EF8-83E4-C680FEA2BC50}"/>
-    <hyperlink ref="C38" r:id="rId46" xr:uid="{58947F88-6578-4261-92AC-CAC9823D178C}"/>
-    <hyperlink ref="C56" r:id="rId47" xr:uid="{F1DEA5CC-77DB-423D-AE92-DDC7B188FA93}"/>
-    <hyperlink ref="C12" r:id="rId48" xr:uid="{996D2E2A-8F47-4EE1-B966-8D058D65D294}"/>
+    <hyperlink ref="C43" r:id="rId25" xr:uid="{3682C2B1-4476-4430-8109-2353A524C137}"/>
+    <hyperlink ref="C52" r:id="rId26" xr:uid="{4E741034-1394-42D0-8739-142B2406FCB0}"/>
+    <hyperlink ref="C45" r:id="rId27" xr:uid="{B384043F-23E3-43F1-862B-A7356F8867EC}"/>
+    <hyperlink ref="C53" r:id="rId28" xr:uid="{6E3DD45A-D91A-4A36-BF25-EEBD7F10DAE9}"/>
+    <hyperlink ref="C54" r:id="rId29" xr:uid="{6453CA4A-2AC9-4105-BF0F-FBCA99EEB8D1}"/>
+    <hyperlink ref="C55" r:id="rId30" xr:uid="{AA389CBE-2BA8-4629-8201-C6131E27DFBE}"/>
+    <hyperlink ref="C57" r:id="rId31" xr:uid="{6F0FC5B8-F6F6-4C15-BB76-EAAC8F1ACA1A}"/>
+    <hyperlink ref="C58" r:id="rId32" xr:uid="{567094FA-4502-4190-8663-26683FDE48C7}"/>
+    <hyperlink ref="C14" r:id="rId33" xr:uid="{A74EF970-0D7C-46E9-AC9F-E64E0416DCED}"/>
+    <hyperlink ref="C15" r:id="rId34" xr:uid="{4119277E-53BD-480A-AAD0-5BF01C147C02}"/>
+    <hyperlink ref="C16" r:id="rId35" xr:uid="{F67B1A2A-4358-43B4-86C7-5A00503AFF4C}"/>
+    <hyperlink ref="C21" r:id="rId36" xr:uid="{D337D021-F911-411B-BC13-9CBEF73345EF}"/>
+    <hyperlink ref="C25" r:id="rId37" xr:uid="{740D5D52-5E21-47B4-AE24-5AD4FADFC13D}"/>
+    <hyperlink ref="C26" r:id="rId38" xr:uid="{1E8B1C6A-A129-4E2E-9CF9-FFC3608F8F60}"/>
+    <hyperlink ref="C27" r:id="rId39" xr:uid="{F9D674A4-D18C-4CA7-BDBD-994C52816696}"/>
+    <hyperlink ref="C30" r:id="rId40" xr:uid="{C0358119-16A3-40A0-ACE5-D9B3CA1113E8}"/>
+    <hyperlink ref="C33" r:id="rId41" xr:uid="{17934D35-BFF5-473B-9CF6-081553A57DB8}"/>
+    <hyperlink ref="C34" r:id="rId42" xr:uid="{C23108EC-6E51-4B52-BFBF-0ECFFE00B2CC}"/>
+    <hyperlink ref="C35" r:id="rId43" xr:uid="{58BEF89A-A2C4-4EF8-83E4-C680FEA2BC50}"/>
+    <hyperlink ref="C38" r:id="rId44" xr:uid="{58947F88-6578-4261-92AC-CAC9823D178C}"/>
+    <hyperlink ref="C56" r:id="rId45" xr:uid="{F1DEA5CC-77DB-423D-AE92-DDC7B188FA93}"/>
+    <hyperlink ref="C12" r:id="rId46" xr:uid="{996D2E2A-8F47-4EE1-B966-8D058D65D294}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>